<commit_message>
Atualização automática - Planilha ReceitaxDespesa
</commit_message>
<xml_diff>
--- a/Grafico_Grupo de Despesa.xlsx
+++ b/Grafico_Grupo de Despesa.xlsx
@@ -2,25 +2,29 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\172.17.1.6\coord_plan_institucional\DADOS CPI\Orçamento\2026\EXECUÇÃO ORÇAMENTÁRIA\RELEXORC_CSV\Saida_PowerBI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Rei-1cpd003\coord_plan_institucional\DADOS CPI\Orçamento\2026\EXECUÇÃO ORÇAMENTÁRIA\RELEXORC_CSV\Saida_PowerBI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19EE4AFB-2C4E-4882-97D3-728CA60F74CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8707B50-AA76-4BE6-B411-F71B4AF47C9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BD803231-520B-43E5-B415-970328918330}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BD803231-520B-43E5-B415-970328918330}"/>
   </bookViews>
   <sheets>
     <sheet name="ReceitaXDespesa" sheetId="3" r:id="rId1"/>
-    <sheet name="Exec_Por Grupo" sheetId="1" state="hidden" r:id="rId2"/>
-    <sheet name="Planilha1" sheetId="2" state="hidden" r:id="rId3"/>
+    <sheet name="Planilha2" sheetId="4" r:id="rId2"/>
+    <sheet name="Exec_Por Grupo" sheetId="1" state="hidden" r:id="rId3"/>
+    <sheet name="Planilha1" sheetId="2" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">Planilha1!$A$1:$P$59</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">Planilha1!$A$1:$P$59</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="1" r:id="rId5"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -268,7 +272,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -330,11 +334,122 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="65"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color indexed="65"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -419,6 +534,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2415,6 +2539,320 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Leopoldo Euler Marialva de Albuquerque" refreshedDate="46275.40976412037" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="53" xr:uid="{96A2F22B-9851-447E-BF55-32AFFD6526E0}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:C1048576" sheet="ReceitaXDespesa"/>
+  </cacheSource>
+  <cacheFields count="3">
+    <cacheField name="Mês/Ano" numFmtId="0">
+      <sharedItems containsNonDate="0" containsDate="1" containsString="0" containsBlank="1" minDate="2026-01-01T00:00:00" maxDate="2026-12-02T00:00:00"/>
+    </cacheField>
+    <cacheField name="Item Orçamentário" numFmtId="0">
+      <sharedItems containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Valor" numFmtId="0">
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="-91.791328169999986" maxValue="154.63542719999998"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="53">
+  <r>
+    <d v="2026-01-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-01-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <n v="62.844099030000002"/>
+  </r>
+  <r>
+    <d v="2026-01-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <n v="154.63542719999998"/>
+  </r>
+  <r>
+    <d v="2026-01-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="-91.791328169999986"/>
+  </r>
+  <r>
+    <d v="2026-02-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-02-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <n v="71.107409860000004"/>
+  </r>
+  <r>
+    <d v="2026-02-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <n v="65.867006619999998"/>
+  </r>
+  <r>
+    <d v="2026-02-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="5.2404032400000062"/>
+  </r>
+  <r>
+    <d v="2026-03-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-03-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <n v="75.044984989999989"/>
+  </r>
+  <r>
+    <d v="2026-03-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <n v="54.581181280000003"/>
+  </r>
+  <r>
+    <d v="2026-03-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="20.463803709999986"/>
+  </r>
+  <r>
+    <d v="2026-04-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-04-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <n v="91.82818374"/>
+  </r>
+  <r>
+    <d v="2026-04-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <n v="41.371067400000001"/>
+  </r>
+  <r>
+    <d v="2026-04-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="50.457116339999999"/>
+  </r>
+  <r>
+    <d v="2026-05-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-05-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <n v="77.415932499999997"/>
+  </r>
+  <r>
+    <d v="2026-05-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <n v="80.184171169999999"/>
+  </r>
+  <r>
+    <d v="2026-05-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="-2.7682386700000023"/>
+  </r>
+  <r>
+    <d v="2026-06-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-06-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <n v="75.166762640000002"/>
+  </r>
+  <r>
+    <d v="2026-06-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <n v="92.382151069999992"/>
+  </r>
+  <r>
+    <d v="2026-06-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="-17.21538842999999"/>
+  </r>
+  <r>
+    <d v="2026-07-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-07-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <n v="70.888043189999991"/>
+  </r>
+  <r>
+    <d v="2026-07-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <n v="99.462564389999997"/>
+  </r>
+  <r>
+    <d v="2026-07-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="-28.574521200000007"/>
+  </r>
+  <r>
+    <d v="2026-08-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-08-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <n v="76.738591329999991"/>
+  </r>
+  <r>
+    <d v="2026-08-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <n v="77.35292192"/>
+  </r>
+  <r>
+    <d v="2026-08-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="-0.61433059000000867"/>
+  </r>
+  <r>
+    <d v="2026-09-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-09-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <m/>
+  </r>
+  <r>
+    <d v="2026-09-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <m/>
+  </r>
+  <r>
+    <d v="2026-09-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="0"/>
+  </r>
+  <r>
+    <d v="2026-10-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-10-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <m/>
+  </r>
+  <r>
+    <d v="2026-10-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <m/>
+  </r>
+  <r>
+    <d v="2026-10-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="0"/>
+  </r>
+  <r>
+    <d v="2026-11-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-11-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <m/>
+  </r>
+  <r>
+    <d v="2026-11-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <m/>
+  </r>
+  <r>
+    <d v="2026-11-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="0"/>
+  </r>
+  <r>
+    <d v="2026-12-01T00:00:00"/>
+    <s v="LOA (A)"/>
+    <n v="84.4166666666667"/>
+  </r>
+  <r>
+    <d v="2026-12-01T00:00:00"/>
+    <s v="Receita Arrecadada (B)"/>
+    <m/>
+  </r>
+  <r>
+    <d v="2026-12-01T00:00:00"/>
+    <s v="Despesa Realizada (C)"/>
+    <m/>
+  </r>
+  <r>
+    <d v="2026-12-01T00:00:00"/>
+    <s v="Saldo (B-C)"/>
+    <n v="0"/>
+  </r>
+  <r>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+  <r>
+    <m/>
+    <m/>
+    <m/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5606F569-D500-4B4F-95B4-2EACD5DAD170}" name="Tabela dinâmica1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A1:C18" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="3">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
@@ -3303,6 +3741,106 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD7906E5-5AAB-4F02-B6BE-5DAC634E0134}">
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="32"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="34"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="35"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="37"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="35"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="37"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="35"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="37"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="35"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="37"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="35"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="37"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="35"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="37"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="35"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="37"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="35"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="37"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="35"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="37"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="35"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="37"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="35"/>
+      <c r="B12" s="36"/>
+      <c r="C12" s="37"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="35"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="37"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="35"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="37"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="35"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="37"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="35"/>
+      <c r="B16" s="36"/>
+      <c r="C16" s="37"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="35"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="37"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="38"/>
+      <c r="B18" s="39"/>
+      <c r="C18" s="40"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89F53F72-D795-49FC-9398-FBDE53A0A7F9}">
   <dimension ref="B3:G28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3430,7 +3968,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDAC02C4-A2C3-4869-A45C-FC4CAB74D8EC}">
   <dimension ref="A2:U59"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>

</xml_diff>